<commit_message>
update det 2.5 benchmark results
</commit_message>
<xml_diff>
--- a/tests/perf_v2/perf_history/v2.5/detection/DETECTION-high-level-summary.xlsx
+++ b/tests/perf_v2/perf_history/v2.5/detection/DETECTION-high-level-summary.xlsx
@@ -613,7 +613,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -623,104 +623,104 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>atss_mobilenetv2</t>
+          <t>atss_resnext101</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>46.7667</v>
+        <v>37.6667</v>
       </c>
       <c r="E2" t="n">
-        <v>16.6044</v>
+        <v>10.8326</v>
       </c>
       <c r="F2" t="n">
-        <v>389.7347</v>
+        <v>1178.9854</v>
       </c>
       <c r="G2" t="n">
-        <v>863.2228</v>
+        <v>2688.9701</v>
       </c>
       <c r="H2" t="n">
-        <v>6.6633</v>
+        <v>15.4582</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2494</v>
+        <v>0.062</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2044</v>
+        <v>0.495</v>
       </c>
       <c r="K2" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.025</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6538</v>
+        <v>0.6857</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1738</v>
+        <v>0.1805</v>
       </c>
       <c r="N2" t="n">
-        <v>0.5521</v>
+        <v>0.5733</v>
       </c>
       <c r="O2" t="n">
-        <v>0.2097</v>
+        <v>0.2236</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1174</v>
+        <v>0.4983</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0752</v>
+        <v>0.0623</v>
       </c>
       <c r="R2" t="n">
-        <v>8.710900000000001</v>
+        <v>41.7895</v>
       </c>
       <c r="S2" t="n">
-        <v>6.3428</v>
+        <v>32.5133</v>
       </c>
       <c r="T2" t="n">
-        <v>0.5727</v>
+        <v>0.6055</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1969</v>
+        <v>0.1965</v>
       </c>
       <c r="V2" t="n">
-        <v>0.1302</v>
+        <v>0.1809</v>
       </c>
       <c r="W2" t="n">
-        <v>0.06710000000000001</v>
+        <v>0.0031</v>
       </c>
       <c r="X2" t="n">
-        <v>0.0581</v>
+        <v>0.0968</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.0238</v>
+        <v>0.0199</v>
       </c>
       <c r="Z2" t="n">
-        <v>4.8117</v>
+        <v>7.9733</v>
       </c>
       <c r="AA2" t="n">
-        <v>4.1663</v>
+        <v>6.4553</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.5508999999999999</v>
+        <v>0.5709</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.2101</v>
+        <v>0.2249</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.1232</v>
+        <v>0.2024</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.0738</v>
+        <v>0.06469999999999999</v>
       </c>
       <c r="AF2" t="n">
-        <v>8.8462</v>
+        <v>15.6063</v>
       </c>
       <c r="AG2" t="n">
-        <v>5.9032</v>
+        <v>10.1128</v>
       </c>
       <c r="AH2" t="n">
-        <v>41.059</v>
+        <v>231.064</v>
       </c>
       <c r="AI2" t="n">
-        <v>31.1338</v>
+        <v>230.2479</v>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -741,104 +741,104 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>atss_resnext101</t>
+          <t>dfine_x</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>39.1</v>
+        <v>55.6667</v>
       </c>
       <c r="E3" t="n">
-        <v>15.3321</v>
+        <v>17.6853</v>
       </c>
       <c r="F3" t="n">
-        <v>808.8727</v>
+        <v>1498.8786</v>
       </c>
       <c r="G3" t="n">
-        <v>1864.9864</v>
+        <v>2299.2035</v>
       </c>
       <c r="H3" t="n">
-        <v>9.8233</v>
+        <v>20.9737</v>
       </c>
       <c r="I3" t="n">
-        <v>0.115</v>
+        <v>0.9641</v>
       </c>
       <c r="J3" t="n">
-        <v>0.302</v>
+        <v>0.8856000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0132</v>
+        <v>0.7654</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6935</v>
+        <v>0.7221</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1633</v>
+        <v>0.144</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5753</v>
+        <v>0.6231</v>
       </c>
       <c r="O3" t="n">
-        <v>0.2186</v>
+        <v>0.1842</v>
       </c>
       <c r="P3" t="n">
-        <v>0.4986</v>
+        <v>0.2404</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.064</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="R3" t="n">
-        <v>41.7855</v>
+        <v>18.9636</v>
       </c>
       <c r="S3" t="n">
-        <v>32.5525</v>
+        <v>13.0572</v>
       </c>
       <c r="T3" t="n">
-        <v>0.607</v>
+        <v>0.6328</v>
       </c>
       <c r="U3" t="n">
-        <v>0.1927</v>
+        <v>0.1823</v>
       </c>
       <c r="V3" t="n">
-        <v>0.1308</v>
+        <v>0.1979</v>
       </c>
       <c r="W3" t="n">
-        <v>0.0063</v>
+        <v>0.1145</v>
       </c>
       <c r="X3" t="n">
-        <v>0.099</v>
+        <v>0.1095</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.0237</v>
+        <v>0.0409</v>
       </c>
       <c r="Z3" t="n">
-        <v>7.818</v>
+        <v>9.3523</v>
       </c>
       <c r="AA3" t="n">
-        <v>5.7042</v>
+        <v>8.955</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.5737</v>
+        <v>0.4039</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.2174</v>
+        <v>0.3257</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.2038</v>
+        <v>0.2215</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0878</v>
       </c>
       <c r="AF3" t="n">
-        <v>15.6981</v>
+        <v>15.8315</v>
       </c>
       <c r="AG3" t="n">
-        <v>10.1593</v>
+        <v>8.3149</v>
       </c>
       <c r="AH3" t="n">
-        <v>244.9802</v>
+        <v>350.3607</v>
       </c>
       <c r="AI3" t="n">
-        <v>228.3143</v>
+        <v>363.9204</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -859,104 +859,104 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>dfine_x</t>
+          <t>rtdetr_101</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>41.9</v>
+        <v>47.1833</v>
       </c>
       <c r="E4" t="n">
-        <v>21.4679</v>
+        <v>13.1684</v>
       </c>
       <c r="F4" t="n">
-        <v>667.9627</v>
+        <v>1511.6825</v>
       </c>
       <c r="G4" t="n">
-        <v>644.1165</v>
+        <v>2165.2491</v>
       </c>
       <c r="H4" t="n">
-        <v>14.7753</v>
+        <v>10.494</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9949</v>
+        <v>0.5833</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8309</v>
+        <v>0.6665</v>
       </c>
       <c r="K4" t="n">
-        <v>0.781</v>
+        <v>0.6979</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6989</v>
+        <v>0.6531</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1515</v>
+        <v>0.1887</v>
       </c>
       <c r="N4" t="n">
-        <v>0.6117</v>
+        <v>0.5452</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1819</v>
+        <v>0.2393</v>
       </c>
       <c r="P4" t="n">
-        <v>0.2399</v>
+        <v>0.2617</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.074</v>
+        <v>0.06660000000000001</v>
       </c>
       <c r="R4" t="n">
-        <v>18.9303</v>
+        <v>21.2434</v>
       </c>
       <c r="S4" t="n">
-        <v>13.0843</v>
+        <v>15.6575</v>
       </c>
       <c r="T4" t="n">
-        <v>0.6307</v>
+        <v>0.5646</v>
       </c>
       <c r="U4" t="n">
-        <v>0.1803</v>
+        <v>0.2295</v>
       </c>
       <c r="V4" t="n">
-        <v>0.1887</v>
+        <v>0.2095</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1277</v>
+        <v>0.1082</v>
       </c>
       <c r="X4" t="n">
-        <v>0.1155</v>
+        <v>0.1132</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.0437</v>
+        <v>0.0409</v>
       </c>
       <c r="Z4" t="n">
-        <v>9.689299999999999</v>
+        <v>9.6676</v>
       </c>
       <c r="AA4" t="n">
-        <v>8.9482</v>
+        <v>9.1572</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.4342</v>
+        <v>0.4773</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.3061</v>
+        <v>0.2656</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.2231</v>
+        <v>0.2162</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.0897</v>
+        <v>0.0876</v>
       </c>
       <c r="AF4" t="n">
-        <v>15.9602</v>
+        <v>16.3924</v>
       </c>
       <c r="AG4" t="n">
-        <v>8.433400000000001</v>
+        <v>11.0637</v>
       </c>
       <c r="AH4" t="n">
-        <v>357.6031</v>
+        <v>123.7221</v>
       </c>
       <c r="AI4" t="n">
-        <v>367.8664</v>
+        <v>85.36069999999999</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -977,104 +977,104 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>rtdetr_101</t>
+          <t>rtdetr_18</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>32.9167</v>
+        <v>52.5167</v>
       </c>
       <c r="E5" t="n">
-        <v>16.4196</v>
+        <v>14.2906</v>
       </c>
       <c r="F5" t="n">
-        <v>707.0263</v>
+        <v>1499.2345</v>
       </c>
       <c r="G5" t="n">
-        <v>826.0271</v>
+        <v>2487.1636</v>
       </c>
       <c r="H5" t="n">
-        <v>9.5932</v>
+        <v>5.5112</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5224</v>
+        <v>0.1373</v>
       </c>
       <c r="J5" t="n">
-        <v>0.6488</v>
+        <v>0.5407</v>
       </c>
       <c r="K5" t="n">
-        <v>0.7155</v>
+        <v>0.7436</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6288</v>
+        <v>0.6211</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1947</v>
+        <v>0.1742</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5153</v>
+        <v>0.4998</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2427</v>
+        <v>0.2449</v>
       </c>
       <c r="P5" t="n">
-        <v>0.2626</v>
+        <v>0.1311</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0701</v>
+        <v>0.0805</v>
       </c>
       <c r="R5" t="n">
-        <v>21.263</v>
+        <v>10.2172</v>
       </c>
       <c r="S5" t="n">
-        <v>15.5834</v>
+        <v>8.1953</v>
       </c>
       <c r="T5" t="n">
-        <v>0.537</v>
+        <v>0.5196</v>
       </c>
       <c r="U5" t="n">
-        <v>0.2361</v>
+        <v>0.2319</v>
       </c>
       <c r="V5" t="n">
-        <v>0.1903</v>
+        <v>0.1628</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1153</v>
+        <v>0.1475</v>
       </c>
       <c r="X5" t="n">
-        <v>0.1213</v>
+        <v>0.0907</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.0426</v>
+        <v>0.0452</v>
       </c>
       <c r="Z5" t="n">
-        <v>10.0698</v>
+        <v>8.085699999999999</v>
       </c>
       <c r="AA5" t="n">
-        <v>8.9884</v>
+        <v>8.726599999999999</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.4446</v>
+        <v>0.4348</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.2513</v>
+        <v>0.2711</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.2109</v>
+        <v>0.1315</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.077</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="AF5" t="n">
-        <v>15.7071</v>
+        <v>9.809900000000001</v>
       </c>
       <c r="AG5" t="n">
-        <v>9.392200000000001</v>
+        <v>7.1736</v>
       </c>
       <c r="AH5" t="n">
-        <v>133.546</v>
+        <v>48.966</v>
       </c>
       <c r="AI5" t="n">
-        <v>101.4551</v>
+        <v>34.0604</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1095,104 +1095,104 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rtdetr_18</t>
+          <t>rtdetr_50</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>31.25</v>
+        <v>47.7167</v>
       </c>
       <c r="E6" t="n">
-        <v>14.3144</v>
+        <v>15.8949</v>
       </c>
       <c r="F6" t="n">
-        <v>572.2556</v>
+        <v>1338.6201</v>
       </c>
       <c r="G6" t="n">
-        <v>790.1321</v>
+        <v>2040.5605</v>
       </c>
       <c r="H6" t="n">
-        <v>3.2522</v>
+        <v>7.7198</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2105</v>
+        <v>0.6121</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5565</v>
+        <v>0.6075</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7544999999999999</v>
+        <v>0.7299</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5783</v>
+        <v>0.659</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1883</v>
+        <v>0.1888</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4689</v>
+        <v>0.575</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2594</v>
+        <v>0.2256</v>
       </c>
       <c r="P6" t="n">
-        <v>0.133</v>
+        <v>0.1849</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0847</v>
+        <v>0.0733</v>
       </c>
       <c r="R6" t="n">
-        <v>10.3805</v>
+        <v>14.5748</v>
       </c>
       <c r="S6" t="n">
-        <v>8.401999999999999</v>
+        <v>10.4937</v>
       </c>
       <c r="T6" t="n">
-        <v>0.4786</v>
+        <v>0.5867</v>
       </c>
       <c r="U6" t="n">
-        <v>0.2566</v>
+        <v>0.2151</v>
       </c>
       <c r="V6" t="n">
-        <v>0.1702</v>
+        <v>0.1775</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1587</v>
+        <v>0.1142</v>
       </c>
       <c r="X6" t="n">
-        <v>0.09420000000000001</v>
+        <v>0.0975</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.0472</v>
+        <v>0.0401</v>
       </c>
       <c r="Z6" t="n">
-        <v>8.3819</v>
+        <v>8.6128</v>
       </c>
       <c r="AA6" t="n">
-        <v>8.9549</v>
+        <v>8.8521</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.3896</v>
+        <v>0.5327</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.2752</v>
+        <v>0.242</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.1414</v>
+        <v>0.1838</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.0974</v>
+        <v>0.0895</v>
       </c>
       <c r="AF6" t="n">
-        <v>10.7979</v>
+        <v>13.4889</v>
       </c>
       <c r="AG6" t="n">
-        <v>9.976599999999999</v>
+        <v>8.4337</v>
       </c>
       <c r="AH6" t="n">
-        <v>53.2384</v>
+        <v>91.6015</v>
       </c>
       <c r="AI6" t="n">
-        <v>33.5278</v>
+        <v>74.5727</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1213,104 +1213,104 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>rtdetr_50</t>
+          <t>ssd_mobilenetv2</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>32.2667</v>
+        <v>78.88330000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>14.1456</v>
+        <v>25.4319</v>
       </c>
       <c r="F7" t="n">
-        <v>669.7916</v>
+        <v>909.0399</v>
       </c>
       <c r="G7" t="n">
-        <v>861.4204</v>
+        <v>1507.9665</v>
       </c>
       <c r="H7" t="n">
-        <v>6.8215</v>
+        <v>10.5565</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5788</v>
+        <v>0.199</v>
       </c>
       <c r="J7" t="n">
-        <v>0.612</v>
+        <v>0.3281</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7326</v>
+        <v>0.3556</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6389</v>
+        <v>0.5758</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2057</v>
+        <v>0.213</v>
       </c>
       <c r="N7" t="n">
-        <v>0.5574</v>
+        <v>0.4644</v>
       </c>
       <c r="O7" t="n">
-        <v>0.2323</v>
+        <v>0.2437</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1862</v>
+        <v>0.0987</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0756</v>
+        <v>0.0779</v>
       </c>
       <c r="R7" t="n">
-        <v>14.6542</v>
+        <v>7.5977</v>
       </c>
       <c r="S7" t="n">
-        <v>10.4585</v>
+        <v>6.668</v>
       </c>
       <c r="T7" t="n">
-        <v>0.5691000000000001</v>
+        <v>0.4835</v>
       </c>
       <c r="U7" t="n">
-        <v>0.2309</v>
+        <v>0.2301</v>
       </c>
       <c r="V7" t="n">
-        <v>0.1816</v>
+        <v>0.1271</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1445</v>
+        <v>0.0718</v>
       </c>
       <c r="X7" t="n">
-        <v>0.1079</v>
+        <v>0.065</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.0455</v>
+        <v>0.0259</v>
       </c>
       <c r="Z7" t="n">
-        <v>9.209300000000001</v>
+        <v>5.8968</v>
       </c>
       <c r="AA7" t="n">
-        <v>8.955399999999999</v>
+        <v>6.249</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.5192</v>
+        <v>0.4628</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.245</v>
+        <v>0.2448</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.19</v>
+        <v>0.0945</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.0998</v>
+        <v>0.0764</v>
       </c>
       <c r="AF7" t="n">
-        <v>14.242</v>
+        <v>7.1454</v>
       </c>
       <c r="AG7" t="n">
-        <v>11.056</v>
+        <v>6.3661</v>
       </c>
       <c r="AH7" t="n">
-        <v>91.20569999999999</v>
+        <v>32.619</v>
       </c>
       <c r="AI7" t="n">
-        <v>65.71769999999999</v>
+        <v>25.524</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1331,104 +1331,104 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>rtmdet_tiny</t>
+          <t>yolox_l</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>69.86669999999999</v>
+        <v>64.58329999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>22.1998</v>
+        <v>19.8599</v>
       </c>
       <c r="F8" t="n">
-        <v>732.3261</v>
+        <v>726.7983</v>
       </c>
       <c r="G8" t="n">
-        <v>1372.4334</v>
+        <v>1473.3412</v>
       </c>
       <c r="H8" t="n">
-        <v>2.0492</v>
+        <v>13.9217</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6884</v>
+        <v>0.8124</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2505</v>
+        <v>0.3319</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2523</v>
+        <v>0.1483</v>
       </c>
       <c r="L8" t="n">
-        <v>0.6328</v>
+        <v>0.6775</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1971</v>
+        <v>0.2034</v>
       </c>
       <c r="N8" t="n">
-        <v>0.5404</v>
+        <v>0.5783</v>
       </c>
       <c r="O8" t="n">
-        <v>0.2254</v>
+        <v>0.246</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1055</v>
+        <v>0.1701</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0896</v>
+        <v>0.067</v>
       </c>
       <c r="R8" t="n">
-        <v>7.7362</v>
+        <v>13.5624</v>
       </c>
       <c r="S8" t="n">
-        <v>6.6327</v>
+        <v>10.0673</v>
       </c>
       <c r="T8" t="n">
-        <v>0.5582</v>
+        <v>0.6038</v>
       </c>
       <c r="U8" t="n">
-        <v>0.2148</v>
+        <v>0.2342</v>
       </c>
       <c r="V8" t="n">
-        <v>0.1413</v>
+        <v>0.1154</v>
       </c>
       <c r="W8" t="n">
-        <v>0.0857</v>
+        <v>0.043</v>
       </c>
       <c r="X8" t="n">
-        <v>0.0801</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.0323</v>
+        <v>0.0292</v>
       </c>
       <c r="Z8" t="n">
-        <v>7.3368</v>
+        <v>6.1595</v>
       </c>
       <c r="AA8" t="n">
-        <v>8.0253</v>
+        <v>6.7029</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.5306</v>
+        <v>0.5769</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.2307</v>
+        <v>0.2458</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.1069</v>
+        <v>0.1376</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.07729999999999999</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="AF8" t="n">
-        <v>7.8129</v>
+        <v>10.0822</v>
       </c>
       <c r="AG8" t="n">
-        <v>6.1179</v>
+        <v>6.8402</v>
       </c>
       <c r="AH8" t="n">
-        <v>25.0616</v>
+        <v>62.3817</v>
       </c>
       <c r="AI8" t="n">
-        <v>14.4447</v>
+        <v>43.3333</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
@@ -1449,104 +1449,104 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ssd_mobilenetv2</t>
+          <t>atss_mobilenetv2</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>81.5667</v>
+        <v>46.7667</v>
       </c>
       <c r="E9" t="n">
-        <v>25.9774</v>
+        <v>16.6044</v>
       </c>
       <c r="F9" t="n">
-        <v>978.7958</v>
+        <v>389.7347</v>
       </c>
       <c r="G9" t="n">
-        <v>1634.6663</v>
+        <v>863.2228</v>
       </c>
       <c r="H9" t="n">
-        <v>5.558</v>
+        <v>6.6633</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2578</v>
+        <v>0.2494</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3068</v>
+        <v>0.2044</v>
       </c>
       <c r="K9" t="n">
-        <v>0.3667</v>
+        <v>0.09710000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5737</v>
+        <v>0.6538</v>
       </c>
       <c r="M9" t="n">
+        <v>0.1738</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.5521</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.2097</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.1174</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.0752</v>
+      </c>
+      <c r="R9" t="n">
+        <v>8.710900000000001</v>
+      </c>
+      <c r="S9" t="n">
+        <v>6.3428</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.5727</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.1969</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.1302</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.06710000000000001</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.0581</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>4.8117</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>4.1663</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.5508999999999999</v>
+      </c>
+      <c r="AC9" t="n">
         <v>0.2101</v>
       </c>
-      <c r="N9" t="n">
-        <v>0.4723</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.2294</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.09950000000000001</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.0751</v>
-      </c>
-      <c r="R9" t="n">
-        <v>7.6786</v>
-      </c>
-      <c r="S9" t="n">
-        <v>6.6724</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.4868</v>
-      </c>
-      <c r="U9" t="n">
-        <v>0.2233</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0.1272</v>
-      </c>
-      <c r="W9" t="n">
-        <v>0.0713</v>
-      </c>
-      <c r="X9" t="n">
-        <v>0.0682</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>0.0252</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>6.0694</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>6.2046</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>0.4723</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>0.2288</v>
-      </c>
       <c r="AD9" t="n">
-        <v>0.0956</v>
+        <v>0.1232</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.0751</v>
+        <v>0.0738</v>
       </c>
       <c r="AF9" t="n">
-        <v>7.2425</v>
+        <v>8.8462</v>
       </c>
       <c r="AG9" t="n">
-        <v>6.3932</v>
+        <v>5.9032</v>
       </c>
       <c r="AH9" t="n">
-        <v>32.1154</v>
+        <v>41.059</v>
       </c>
       <c r="AI9" t="n">
-        <v>25.6519</v>
+        <v>31.1338</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
@@ -1567,104 +1567,104 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>yolox_l</t>
+          <t>rtmdet_tiny</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>60.7667</v>
+        <v>69.86669999999999</v>
       </c>
       <c r="E10" t="n">
-        <v>17.4651</v>
+        <v>22.1998</v>
       </c>
       <c r="F10" t="n">
-        <v>647.14</v>
+        <v>732.3261</v>
       </c>
       <c r="G10" t="n">
-        <v>1283.9758</v>
+        <v>1372.4334</v>
       </c>
       <c r="H10" t="n">
-        <v>8.046799999999999</v>
+        <v>2.0492</v>
       </c>
       <c r="I10" t="n">
-        <v>1.3057</v>
+        <v>0.6884</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2641</v>
+        <v>0.2505</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1738</v>
+        <v>0.2523</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6781</v>
+        <v>0.6328</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1961</v>
+        <v>0.1971</v>
       </c>
       <c r="N10" t="n">
-        <v>0.5752</v>
+        <v>0.5404</v>
       </c>
       <c r="O10" t="n">
-        <v>0.2427</v>
+        <v>0.2254</v>
       </c>
       <c r="P10" t="n">
-        <v>0.1699</v>
+        <v>0.1055</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.0665</v>
+        <v>0.0896</v>
       </c>
       <c r="R10" t="n">
-        <v>13.6496</v>
+        <v>7.7362</v>
       </c>
       <c r="S10" t="n">
-        <v>10.344</v>
+        <v>6.6327</v>
       </c>
       <c r="T10" t="n">
-        <v>0.5931</v>
+        <v>0.5582</v>
       </c>
       <c r="U10" t="n">
-        <v>0.2417</v>
+        <v>0.2148</v>
       </c>
       <c r="V10" t="n">
-        <v>0.1179</v>
+        <v>0.1413</v>
       </c>
       <c r="W10" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.0857</v>
       </c>
       <c r="X10" t="n">
-        <v>0.0828</v>
+        <v>0.0801</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.0349</v>
+        <v>0.0323</v>
       </c>
       <c r="Z10" t="n">
-        <v>6.9896</v>
+        <v>7.3368</v>
       </c>
       <c r="AA10" t="n">
-        <v>6.6926</v>
+        <v>8.0253</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.5707</v>
+        <v>0.5306</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.2425</v>
+        <v>0.2307</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.1383</v>
+        <v>0.1069</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.0794</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="AF10" t="n">
-        <v>10.1631</v>
+        <v>7.8129</v>
       </c>
       <c r="AG10" t="n">
-        <v>7.0032</v>
+        <v>6.1179</v>
       </c>
       <c r="AH10" t="n">
-        <v>61.1833</v>
+        <v>25.0616</v>
       </c>
       <c r="AI10" t="n">
-        <v>42.4932</v>
+        <v>14.4447</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>

</xml_diff>